<commit_message>
Risorsa 18 Roadmap: adattata da 24 a 12 mesi (Q1-Q4, Gantt M1-M12)
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risorse/Risorsa_18_Roadmap_24_Mesi.xlsx
+++ b/risorse/Risorsa_18_Roadmap_24_Mesi.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -496,7 +496,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI Osha — Risorsa 16 · Roadmap AI 24 Mesi</t>
+          <t>AI Osha — Risorsa 18 · Roadmap AI 12 Mesi</t>
         </is>
       </c>
     </row>
@@ -710,173 +710,13 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Q5 (mesi 13-15)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Automazioni</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>Primi 2 agenti AI</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Workflow lead-routing, agente estrai-dati da fatture</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>IT / Operations</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>1500</v>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>2 agenti in produzione; ROI &gt; 3x</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Q6 (mesi 16-18)</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Policy e ruoli</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Pubblicazione policy AI, formazione compliance, audit semestrale</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>Direzione</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>400</v>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>100% staff firma la policy; 0 incidenti AI</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Q7 (mesi 19-21)</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Vantaggio competitivo</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Differenziazione di mercato</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Servizio potenziato con AI per i clienti, case study pubblici</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Direzione + Marketing</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>1200</v>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>1 servizio AI lanciato; +10% lead inbound</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>Q8 (mesi 22-24)</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Scala</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Sistematizzazione e miglioramento</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Review dell'intero stack, retraining team, roadmap anno 3</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>Tutto il team</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>800</v>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>Uso AI &gt; 60%; NPS interno &gt; 8</t>
-        </is>
-      </c>
-      <c r="H12" s="6" t="inlineStr">
-        <is>
-          <t>Da fare</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>BUDGET TOTALE 24 MESI</t>
-        </is>
-      </c>
-      <c r="F13" s="7">
-        <f>SUM(F5:F12)</f>
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>BUDGET TOTALE 12 MESI</t>
+        </is>
+      </c>
+      <c r="F9" s="7">
+        <f>SUM(F5:F8)</f>
         <v/>
       </c>
     </row>
@@ -891,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y12"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -924,7 +764,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>AI Osha — Gantt visivo 24 mesi</t>
+          <t>AI Osha — Gantt visivo 12 mesi</t>
         </is>
       </c>
     </row>
@@ -999,66 +839,6 @@
       <c r="M4" s="9" t="inlineStr">
         <is>
           <t>M12</t>
-        </is>
-      </c>
-      <c r="N4" s="9" t="inlineStr">
-        <is>
-          <t>M13</t>
-        </is>
-      </c>
-      <c r="O4" s="9" t="inlineStr">
-        <is>
-          <t>M14</t>
-        </is>
-      </c>
-      <c r="P4" s="9" t="inlineStr">
-        <is>
-          <t>M15</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>M16</t>
-        </is>
-      </c>
-      <c r="R4" s="9" t="inlineStr">
-        <is>
-          <t>M17</t>
-        </is>
-      </c>
-      <c r="S4" s="9" t="inlineStr">
-        <is>
-          <t>M18</t>
-        </is>
-      </c>
-      <c r="T4" s="9" t="inlineStr">
-        <is>
-          <t>M19</t>
-        </is>
-      </c>
-      <c r="U4" s="9" t="inlineStr">
-        <is>
-          <t>M20</t>
-        </is>
-      </c>
-      <c r="V4" s="9" t="inlineStr">
-        <is>
-          <t>M21</t>
-        </is>
-      </c>
-      <c r="W4" s="9" t="inlineStr">
-        <is>
-          <t>M22</t>
-        </is>
-      </c>
-      <c r="X4" s="9" t="inlineStr">
-        <is>
-          <t>M23</t>
-        </is>
-      </c>
-      <c r="Y4" s="9" t="inlineStr">
-        <is>
-          <t>M24</t>
         </is>
       </c>
     </row>
@@ -1101,46 +881,6 @@
       <c r="K8" s="10" t="n"/>
       <c r="L8" s="10" t="n"/>
       <c r="M8" s="10" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Automazioni</t>
-        </is>
-      </c>
-      <c r="N9" s="10" t="n"/>
-      <c r="O9" s="10" t="n"/>
-      <c r="P9" s="10" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Governance</t>
-        </is>
-      </c>
-      <c r="Q10" s="10" t="n"/>
-      <c r="R10" s="10" t="n"/>
-      <c r="S10" s="10" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Vantaggio competitivo</t>
-        </is>
-      </c>
-      <c r="T11" s="10" t="n"/>
-      <c r="U11" s="10" t="n"/>
-      <c r="V11" s="10" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Scala</t>
-        </is>
-      </c>
-      <c r="W12" s="10" t="n"/>
-      <c r="X12" s="10" t="n"/>
-      <c r="Y12" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>